<commit_message>
chore: Clean up code comments and formatting across multiple files
</commit_message>
<xml_diff>
--- a/Extra/Test_Case.xlsx
+++ b/Extra/Test_Case.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/07c1b08ee16acfbd/Tài liệu/UTH (ws)/LapTrinhMang/012012301310_Group04_UDM09/Extra/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{4E78D9B8-951F-426F-81B6-65880515FBC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0147BBD9-4CE7-43BA-A37A-170316BAC590}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{4E78D9B8-951F-426F-81B6-65880515FBC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C219A2D-5578-474A-971F-48B683F586D4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D6611C0B-3BBD-46A5-A1A3-11670D932E80}"/>
   </bookViews>
@@ -616,6 +616,74 @@
     <dxf>
       <font>
         <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color rgb="FF595959"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -646,6 +714,193 @@
         </bottom>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -685,6 +940,131 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <strike val="0"/>
@@ -716,6 +1096,38 @@
         </bottom>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FFE0E0E0"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FFE0E0E0"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -753,418 +1165,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FFE0E0E0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FFE0E0E0"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color rgb="FF595959"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1179,32 +1179,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{24F15810-B474-4500-A07B-B313BBFDD80A}" name="Table1" displayName="Table1" ref="A1:G15" totalsRowShown="0" headerRowDxfId="1" dataDxfId="12" headerRowBorderDxfId="21" tableBorderDxfId="22" totalsRowBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{24F15810-B474-4500-A07B-B313BBFDD80A}" name="Table1" displayName="Table1" ref="A1:G15" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
   <autoFilter ref="A1:G15" xr:uid="{24F15810-B474-4500-A07B-B313BBFDD80A}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{422ED447-79CB-4FD2-B732-CF8370FA8B91}" name="STT" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{678C89A4-9677-4ABE-9606-D4ADF92DE684}" name="Tên Kịch Bản Kiểm Thử" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{35CB1E03-F9F9-4103-9E13-39231C9F4769}" name="Điều Kiện Ban Đầu" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{BDDDDA38-9E84-4487-A8FF-751704375F39}" name="Các Bước Thực Hiện Kịch Bản" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{4841F281-2B14-453F-88C0-DEC789960F3D}" name="Kết Quả Mong Đợi " dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{085C937C-ADD4-40E4-AF2F-3373934ADDB3}" name="Trạng Thái (P/F)" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{AAA02983-7BC5-479A-A64E-E4E8136F99CB}" name="Ghi Chú" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{422ED447-79CB-4FD2-B732-CF8370FA8B91}" name="STT" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{678C89A4-9677-4ABE-9606-D4ADF92DE684}" name="Tên Kịch Bản Kiểm Thử" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{35CB1E03-F9F9-4103-9E13-39231C9F4769}" name="Điều Kiện Ban Đầu" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{BDDDDA38-9E84-4487-A8FF-751704375F39}" name="Các Bước Thực Hiện Kịch Bản" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{4841F281-2B14-453F-88C0-DEC789960F3D}" name="Kết Quả Mong Đợi " dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{085C937C-ADD4-40E4-AF2F-3373934ADDB3}" name="Trạng Thái (P/F)" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{AAA02983-7BC5-479A-A64E-E4E8136F99CB}" name="Ghi Chú" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D79167D-E7AE-4C7E-91E8-9225ECFB0E9C}" name="Table3" displayName="Table3" ref="A1:G15" totalsRowShown="0" headerRowDxfId="3" dataDxfId="4" headerRowBorderDxfId="10" tableBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D79167D-E7AE-4C7E-91E8-9225ECFB0E9C}" name="Table3" displayName="Table3" ref="A1:G15" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19">
   <autoFilter ref="A1:G15" xr:uid="{3D79167D-E7AE-4C7E-91E8-9225ECFB0E9C}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{5C9B5FB6-C3B7-4787-BE83-963B5EFBD546}" name="STT" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{2DEBF96D-B05C-4914-B3B9-F8DBE1F94E10}" name="Tên Test Case" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{51B984D8-FD8C-4479-B6A4-DF36AE740BA7}" name="Người thực thi" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{87DB0489-3F66-4C12-8889-7B5844CB4433}" name="Ngày thực thi" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{93505694-8F2D-4BD0-8CDA-AD4CFDFC7092}" name="Kết quả thực tế" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{D34F677A-76CA-4D58-BDDC-0FD853BB2D6E}" name="Trạng thái (P/F)" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{790D78E0-D16F-43D9-B19B-5192342B085D}" name="Tên file Proof / Ghi chú" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{5C9B5FB6-C3B7-4787-BE83-963B5EFBD546}" name="STT" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{2DEBF96D-B05C-4914-B3B9-F8DBE1F94E10}" name="Tên Test Case" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{51B984D8-FD8C-4479-B6A4-DF36AE740BA7}" name="Người thực thi" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{87DB0489-3F66-4C12-8889-7B5844CB4433}" name="Ngày thực thi" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{93505694-8F2D-4BD0-8CDA-AD4CFDFC7092}" name="Kết quả thực tế" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{D34F677A-76CA-4D58-BDDC-0FD853BB2D6E}" name="Trạng thái (P/F)" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{790D78E0-D16F-43D9-B19B-5192342B085D}" name="Tên file Proof / Ghi chú" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1874,7 +1874,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
         <v>5</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1890,7 +1890,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
         <v>15</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>25</v>
       </c>
@@ -1914,7 +1914,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="67.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>35</v>
       </c>
@@ -1930,7 +1930,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
@@ -1938,7 +1938,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="67.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>45</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>50</v>
       </c>
@@ -1954,7 +1954,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>55</v>
       </c>
@@ -1962,7 +1962,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -1970,7 +1970,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="67.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>65</v>
       </c>
@@ -1978,7 +1978,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="67.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>70</v>
       </c>

</xml_diff>

<commit_message>
hoàn thành test case 1,2,3
</commit_message>
<xml_diff>
--- a/Extra/Test_Case.xlsx
+++ b/Extra/Test_Case.xlsx
@@ -1,39 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/07c1b08ee16acfbd/Tài liệu/UTH (ws)/LapTrinhMang/012012301310_Group04_UDM09/Extra/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P2P\012012301310_Group04_UDM09\Extra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{4E78D9B8-951F-426F-81B6-65880515FBC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C219A2D-5578-474A-971F-48B683F586D4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{168D3BFE-141E-498D-86FD-36E9D6C43D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D6611C0B-3BBD-46A5-A1A3-11670D932E80}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D6611C0B-3BBD-46A5-A1A3-11670D932E80}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Case" sheetId="1" r:id="rId1"/>
-    <sheet name="Proof" sheetId="2" r:id="rId2"/>
+    <sheet name="TC_01" sheetId="3" r:id="rId2"/>
+    <sheet name="TC_02" sheetId="4" r:id="rId3"/>
+    <sheet name="Proof" sheetId="2" r:id="rId4"/>
+    <sheet name="TC_03" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Case'!$A$1:$G$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -43,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="94">
   <si>
     <t>Tên Kịch Bản Kiểm Thử</t>
   </si>
@@ -346,12 +338,45 @@
   <si>
     <t>Trạng Thái (P/F)</t>
   </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Case A: Bỏ trống cả IP và Port</t>
+  </si>
+  <si>
+    <t>Case B:  Nhập IP đúng, nhập Port ngoài dải biên (0, 65536, -1, 'abc').</t>
+  </si>
+  <si>
+    <t>Case C: Nhập IP sai định dạng phân đoạn (khác IPv4 chuẩn) và Port hợp lệ.</t>
+  </si>
+  <si>
+    <t>Trần Thị Thanh Thơ</t>
+  </si>
+  <si>
+    <t>TC_01!A1</t>
+  </si>
+  <si>
+    <t>TC_02!A1</t>
+  </si>
+  <si>
+    <t>TC_03!A1</t>
+  </si>
+  <si>
+    <t>Ứng dụng khởi động thành công. Thư mục data được tạo tự động (nếu đã xóa trước đó). Không xuất hiện lỗi trong Terminal.</t>
+  </si>
+  <si>
+    <t>Khi cổng 12000 đã bị chiếm, ứng dụng không thể bind vào cổng và hiển thị thông báo "Could not bind to port 12000." trên giao diện. Ứng dụng không bị treo và vẫn phản hồi.</t>
+  </si>
+  <si>
+    <t>Hệ thống từ chối dữ liệu đầu vào không hợp lệ, hiển thị thông báo lỗi và không thực hiện kết nối. Giao diện vẫn hoạt động bình thường.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -396,6 +421,29 @@
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="163"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -557,10 +605,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -608,336 +657,29 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
+    <cellStyle name="Siêu kết nối" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="23">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color rgb="FF595959"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="13"/>
-        <color theme="0"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F4E79"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1165,6 +907,331 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color rgb="FF595959"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFD9D9D9"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FFD9D9D9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="0"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF1F4E79"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1178,33 +1245,946 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>167945</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>8137</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{881C8710-DDF7-400C-800F-81293638B1BA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="3520745" cy="5966977"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>259671</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>145223</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Hình ảnh 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B1972EEC-8298-4BDE-8AB7-E4CCDCF2EAA9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4168140" y="289560"/>
+          <a:ext cx="6820491" cy="5113463"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>186905</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>40772</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0BA33053-E824-453D-B582-DD19A1F9DCE5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="10998679" cy="3663866"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>603850</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>71885</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>230039</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>21286</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Hình ảnh 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8AD7D6B6-00F9-45AA-B2BC-604D88E7E7FD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12091359" y="71885"/>
+          <a:ext cx="9086491" cy="5642835"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>167569</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>560717</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>43030</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Hình ảnh 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{506F698C-11A1-4B4E-BBB0-35D01205071A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="4135720"/>
+          <a:ext cx="11372491" cy="5913952"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>456605</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>89487</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>611273</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>115018</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Hình ảnh 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B905D134-6ED5-43CA-89D3-D7AB8845CA3B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11944114" y="5955449"/>
+          <a:ext cx="6912027" cy="3476097"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>586965</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>53533</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Hình ảnh 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E3608A8-80A8-46C4-A5C2-0D22D697EE29}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="1158240"/>
+          <a:ext cx="2598645" cy="2225233"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>610450</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>91579</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Hình ảnh 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1D729AF-741F-4025-820D-D2D0F2E4446D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2872740" y="1470660"/>
+          <a:ext cx="9807790" cy="1600339"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>403860</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>534167</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>114419</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Hình ảnh 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{168BC97F-3683-481D-ACD7-47A4D3F2D49F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3086100" y="14866620"/>
+          <a:ext cx="8847587" cy="1371719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>22860</xdr:colOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>564101</xdr:colOff>
+      <xdr:row>94</xdr:row>
+      <xdr:rowOff>30640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Hình ảnh 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77A6852D-DBD5-4809-90EF-C32231E95C7D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22860" y="14653260"/>
+          <a:ext cx="2552921" cy="1851820"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>518379</xdr:colOff>
+      <xdr:row>108</xdr:row>
+      <xdr:rowOff>152570</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Hình ảnh 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{38D66324-55C5-4331-B11D-61FC5A0E20F6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7620" y="17114520"/>
+          <a:ext cx="2522439" cy="1966130"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>373380</xdr:colOff>
+      <xdr:row>98</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>107</xdr:row>
+      <xdr:rowOff>33666</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Hình ảnh 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1BE7CCD5-4435-411C-99AB-C0A57D5E9DDD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3055620" y="17586960"/>
+          <a:ext cx="9098280" cy="1611006"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>442173</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>38259</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Hình ảnh 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{73DE4938-E980-46C4-9DB1-AA0A8A5A0991}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="4335780"/>
+          <a:ext cx="2453853" cy="1836579"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>137160</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>221743</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>91563</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Hình ảnh 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF8D9877-C850-4AEC-AC28-55B6E2EC0835}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2819400" y="4625340"/>
+          <a:ext cx="8801863" cy="1425063"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>45949</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>68779</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Hình ảnh 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{92FFEC2F-7BAA-495D-AFE5-CBCBD0A26192}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="83820" y="6355080"/>
+          <a:ext cx="2644369" cy="2301439"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>365760</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>290367</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>152557</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Hình ảnh 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0F44533F-8295-4C0C-ABDA-5D5B70C1401D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3048000" y="6583680"/>
+          <a:ext cx="9312447" cy="1806097"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>564103</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>30656</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Hình ảnh 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7500AED-93BD-419A-A0E1-31BF18DC9D95}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="9044940"/>
+          <a:ext cx="2575783" cy="2027096"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>365760</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>358953</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>15369</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Hình ảnh 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F778AD9-C3D5-4CB0-BD42-5665F7C02C2D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3048000" y="9212580"/>
+          <a:ext cx="9381033" cy="1493649"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>449793</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>53498</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Hình ảnh 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E83C39A2-8629-4AE1-B025-DC73E44C2734}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="11544300"/>
+          <a:ext cx="2461473" cy="1828958"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>84598</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>167770</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Hình ảnh 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B7780DEF-D2C7-44D1-B96F-85CB24064A9D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3177540" y="11811000"/>
+          <a:ext cx="8977138" cy="1501270"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{24F15810-B474-4500-A07B-B313BBFDD80A}" name="Table1" displayName="Table1" ref="A1:G15" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{24F15810-B474-4500-A07B-B313BBFDD80A}" name="Table1" displayName="Table1" ref="A1:G15" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19" totalsRowBorderDxfId="18">
   <autoFilter ref="A1:G15" xr:uid="{24F15810-B474-4500-A07B-B313BBFDD80A}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{422ED447-79CB-4FD2-B732-CF8370FA8B91}" name="STT" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{678C89A4-9677-4ABE-9606-D4ADF92DE684}" name="Tên Kịch Bản Kiểm Thử" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{35CB1E03-F9F9-4103-9E13-39231C9F4769}" name="Điều Kiện Ban Đầu" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{BDDDDA38-9E84-4487-A8FF-751704375F39}" name="Các Bước Thực Hiện Kịch Bản" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{4841F281-2B14-453F-88C0-DEC789960F3D}" name="Kết Quả Mong Đợi " dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{085C937C-ADD4-40E4-AF2F-3373934ADDB3}" name="Trạng Thái (P/F)" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{AAA02983-7BC5-479A-A64E-E4E8136F99CB}" name="Ghi Chú" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{422ED447-79CB-4FD2-B732-CF8370FA8B91}" name="STT" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{678C89A4-9677-4ABE-9606-D4ADF92DE684}" name="Tên Kịch Bản Kiểm Thử" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{35CB1E03-F9F9-4103-9E13-39231C9F4769}" name="Điều Kiện Ban Đầu" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{BDDDDA38-9E84-4487-A8FF-751704375F39}" name="Các Bước Thực Hiện Kịch Bản" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{4841F281-2B14-453F-88C0-DEC789960F3D}" name="Kết Quả Mong Đợi " dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{085C937C-ADD4-40E4-AF2F-3373934ADDB3}" name="Trạng Thái (P/F)" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{AAA02983-7BC5-479A-A64E-E4E8136F99CB}" name="Ghi Chú" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D79167D-E7AE-4C7E-91E8-9225ECFB0E9C}" name="Table3" displayName="Table3" ref="A1:G15" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D79167D-E7AE-4C7E-91E8-9225ECFB0E9C}" name="Table3" displayName="Table3" ref="A1:G15" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7">
   <autoFilter ref="A1:G15" xr:uid="{3D79167D-E7AE-4C7E-91E8-9225ECFB0E9C}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{5C9B5FB6-C3B7-4787-BE83-963B5EFBD546}" name="STT" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{2DEBF96D-B05C-4914-B3B9-F8DBE1F94E10}" name="Tên Test Case" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{51B984D8-FD8C-4479-B6A4-DF36AE740BA7}" name="Người thực thi" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{87DB0489-3F66-4C12-8889-7B5844CB4433}" name="Ngày thực thi" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{93505694-8F2D-4BD0-8CDA-AD4CFDFC7092}" name="Kết quả thực tế" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{D34F677A-76CA-4D58-BDDC-0FD853BB2D6E}" name="Trạng thái (P/F)" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{790D78E0-D16F-43D9-B19B-5192342B085D}" name="Tên file Proof / Ghi chú" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{5C9B5FB6-C3B7-4787-BE83-963B5EFBD546}" name="STT" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{2DEBF96D-B05C-4914-B3B9-F8DBE1F94E10}" name="Tên Test Case" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{51B984D8-FD8C-4479-B6A4-DF36AE740BA7}" name="Người thực thi" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{87DB0489-3F66-4C12-8889-7B5844CB4433}" name="Ngày thực thi" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{93505694-8F2D-4BD0-8CDA-AD4CFDFC7092}" name="Kết quả thực tế" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{D34F677A-76CA-4D58-BDDC-0FD853BB2D6E}" name="Trạng thái (P/F)" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{790D78E0-D16F-43D9-B19B-5192342B085D}" name="Tên file Proof / Ghi chú" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1528,19 +2508,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{265B56AC-4361-4B99-BC23-63B2B2CDA50A}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="16.8"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="64.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.8984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="64.19921875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="65" style="1" customWidth="1"/>
-    <col min="6" max="6" width="24.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="6" max="6" width="24.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.69921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.8984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" s="14" t="s">
         <v>75</v>
       </c>
@@ -1563,7 +2543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" s="5" customFormat="1" ht="100.8">
       <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
@@ -1579,10 +2559,12 @@
       <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="4"/>
+      <c r="F2" s="17" t="s">
+        <v>83</v>
+      </c>
       <c r="G2" s="7"/>
     </row>
-    <row r="3" spans="1:7" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" s="5" customFormat="1" ht="84">
       <c r="A3" s="6" t="s">
         <v>10</v>
       </c>
@@ -1598,10 +2580,12 @@
       <c r="E3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="4"/>
+      <c r="F3" s="17" t="s">
+        <v>83</v>
+      </c>
       <c r="G3" s="7"/>
     </row>
-    <row r="4" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" s="5" customFormat="1" ht="117.6">
       <c r="A4" s="6" t="s">
         <v>15</v>
       </c>
@@ -1617,10 +2601,12 @@
       <c r="E4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="4"/>
+      <c r="F4" s="17" t="s">
+        <v>83</v>
+      </c>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" spans="1:7" s="5" customFormat="1" ht="151.19999999999999" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" s="5" customFormat="1" ht="134.4">
       <c r="A5" s="6" t="s">
         <v>20</v>
       </c>
@@ -1639,7 +2625,7 @@
       <c r="F5" s="4"/>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" s="5" customFormat="1" ht="117.6">
       <c r="A6" s="6" t="s">
         <v>25</v>
       </c>
@@ -1658,7 +2644,7 @@
       <c r="F6" s="4"/>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" spans="1:7" s="5" customFormat="1" ht="134.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" s="5" customFormat="1" ht="134.4">
       <c r="A7" s="6" t="s">
         <v>30</v>
       </c>
@@ -1677,7 +2663,7 @@
       <c r="F7" s="4"/>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" s="5" customFormat="1" ht="117.6">
       <c r="A8" s="6" t="s">
         <v>35</v>
       </c>
@@ -1696,7 +2682,7 @@
       <c r="F8" s="4"/>
       <c r="G8" s="7"/>
     </row>
-    <row r="9" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" s="5" customFormat="1" ht="117.6">
       <c r="A9" s="6" t="s">
         <v>40</v>
       </c>
@@ -1715,7 +2701,7 @@
       <c r="F9" s="4"/>
       <c r="G9" s="7"/>
     </row>
-    <row r="10" spans="1:7" s="5" customFormat="1" ht="134.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" s="5" customFormat="1" ht="100.8">
       <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
@@ -1734,7 +2720,7 @@
       <c r="F10" s="4"/>
       <c r="G10" s="7"/>
     </row>
-    <row r="11" spans="1:7" s="5" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" s="5" customFormat="1" ht="134.4">
       <c r="A11" s="6" t="s">
         <v>50</v>
       </c>
@@ -1753,7 +2739,7 @@
       <c r="F11" s="4"/>
       <c r="G11" s="7"/>
     </row>
-    <row r="12" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" s="5" customFormat="1" ht="100.8">
       <c r="A12" s="6" t="s">
         <v>55</v>
       </c>
@@ -1772,7 +2758,7 @@
       <c r="F12" s="4"/>
       <c r="G12" s="7"/>
     </row>
-    <row r="13" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" s="5" customFormat="1" ht="117.6">
       <c r="A13" s="6" t="s">
         <v>60</v>
       </c>
@@ -1791,7 +2777,7 @@
       <c r="F13" s="4"/>
       <c r="G13" s="7"/>
     </row>
-    <row r="14" spans="1:7" s="5" customFormat="1" ht="134.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" s="5" customFormat="1" ht="117.6">
       <c r="A14" s="6" t="s">
         <v>65</v>
       </c>
@@ -1810,7 +2796,7 @@
       <c r="F14" s="4"/>
       <c r="G14" s="7"/>
     </row>
-    <row r="15" spans="1:7" s="5" customFormat="1" ht="134.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" s="5" customFormat="1" ht="117.6">
       <c r="A15" s="8" t="s">
         <v>70</v>
       </c>
@@ -1838,20 +2824,41 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2740FEBB-4741-4DF0-A699-0C7B375BBE03}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{168DB4B3-5DF8-4A41-93E0-CE7F8314E965}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6E890A5-A39F-47F1-9197-F34001BFD460}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="16.8"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.21875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="23.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="10.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.19921875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.59765625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.8984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.8984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" s="12" t="s">
         <v>75</v>
       </c>
@@ -1874,31 +2881,76 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="50.4">
       <c r="A2" s="13" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C2" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2" s="23">
+        <v>46203</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="F2" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="67.2">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="C3" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="23">
+        <v>46203</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="50.4">
       <c r="A4" s="13" t="s">
         <v>15</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="C4" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="23">
+        <v>46203</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="G4" s="22" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1906,7 +2958,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="33.6">
       <c r="A6" s="13" t="s">
         <v>25</v>
       </c>
@@ -1914,7 +2966,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7">
       <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
@@ -1922,7 +2974,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="33.6">
       <c r="A8" s="13" t="s">
         <v>35</v>
       </c>
@@ -1930,7 +2982,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="33.6">
       <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
@@ -1938,7 +2990,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="33.6">
       <c r="A10" s="13" t="s">
         <v>45</v>
       </c>
@@ -1946,7 +2998,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7">
       <c r="A11" s="2" t="s">
         <v>50</v>
       </c>
@@ -1954,7 +3006,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7">
       <c r="A12" s="13" t="s">
         <v>55</v>
       </c>
@@ -1962,7 +3014,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="33.6">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -1970,7 +3022,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="33.6">
       <c r="A14" s="13" t="s">
         <v>65</v>
       </c>
@@ -1978,7 +3030,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="33.6">
       <c r="A15" s="2" t="s">
         <v>70</v>
       </c>
@@ -1987,9 +3039,41 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" location="TC_01!A1" display="TC_01!A1" xr:uid="{6FC5B747-6378-428C-956E-F75969F1B1D8}"/>
+    <hyperlink ref="G3" location="TC_02!A1" display="TC_02!A1" xr:uid="{EF23B9A1-CF8B-4EB3-8843-CC73EDD3BA1D}"/>
+    <hyperlink ref="G4" location="TC_03!A1" display="TC_03!A1" xr:uid="{DC790DAE-3673-415A-AD8F-1D30E70F15B1}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED1CF396-0CEE-423B-9F0A-D9AA10B67D4E}">
+  <dimension ref="A5:A82"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetData>
+    <row r="5" spans="1:1" ht="24.6">
+      <c r="A5" s="18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="24.6">
+      <c r="A23" s="19" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" ht="24.6">
+      <c r="A82" s="18" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update test case Excel file
</commit_message>
<xml_diff>
--- a/Extra/Test_Case.xlsx
+++ b/Extra/Test_Case.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\P2P\012012301310_Group04_UDM09\Extra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/07c1b08ee16acfbd/Tài liệu/UTH (ws)/LapTrinhMang/012012301310_Group04_UDM09/Extra/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{168D3BFE-141E-498D-86FD-36E9D6C43D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{168D3BFE-141E-498D-86FD-36E9D6C43D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02B95F2E-9261-490D-B0D4-91944B911C37}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D6611C0B-3BBD-46A5-A1A3-11670D932E80}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Case" sheetId="1" r:id="rId1"/>
-    <sheet name="TC_01" sheetId="3" r:id="rId2"/>
-    <sheet name="TC_02" sheetId="4" r:id="rId3"/>
-    <sheet name="Proof" sheetId="2" r:id="rId4"/>
+    <sheet name="Proof" sheetId="2" r:id="rId2"/>
+    <sheet name="TC_01" sheetId="3" r:id="rId3"/>
+    <sheet name="TC_02" sheetId="4" r:id="rId4"/>
     <sheet name="TC_03" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
@@ -376,7 +376,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -676,8 +676,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
-    <cellStyle name="Siêu kết nối" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="23">
     <dxf>
@@ -2508,19 +2508,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{265B56AC-4361-4B99-BC23-63B2B2CDA50A}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="16.8"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.8984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="64.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="64.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="65" style="1" customWidth="1"/>
-    <col min="6" max="6" width="24.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.69921875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.8984375" style="1"/>
+    <col min="6" max="6" width="24.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>75</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="5" customFormat="1" ht="100.8">
+    <row r="2" spans="1:7" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="G2" s="7"/>
     </row>
-    <row r="3" spans="1:7" s="5" customFormat="1" ht="84">
+    <row r="3" spans="1:7" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>10</v>
       </c>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="G3" s="7"/>
     </row>
-    <row r="4" spans="1:7" s="5" customFormat="1" ht="117.6">
+    <row r="4" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>15</v>
       </c>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" spans="1:7" s="5" customFormat="1" ht="134.4">
+    <row r="5" spans="1:7" s="5" customFormat="1" ht="151.19999999999999" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>20</v>
       </c>
@@ -2625,7 +2625,7 @@
       <c r="F5" s="4"/>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="1:7" s="5" customFormat="1" ht="117.6">
+    <row r="6" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>25</v>
       </c>
@@ -2644,7 +2644,7 @@
       <c r="F6" s="4"/>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" spans="1:7" s="5" customFormat="1" ht="134.4">
+    <row r="7" spans="1:7" s="5" customFormat="1" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>30</v>
       </c>
@@ -2663,7 +2663,7 @@
       <c r="F7" s="4"/>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="1:7" s="5" customFormat="1" ht="117.6">
+    <row r="8" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>35</v>
       </c>
@@ -2682,7 +2682,7 @@
       <c r="F8" s="4"/>
       <c r="G8" s="7"/>
     </row>
-    <row r="9" spans="1:7" s="5" customFormat="1" ht="117.6">
+    <row r="9" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>40</v>
       </c>
@@ -2701,7 +2701,7 @@
       <c r="F9" s="4"/>
       <c r="G9" s="7"/>
     </row>
-    <row r="10" spans="1:7" s="5" customFormat="1" ht="100.8">
+    <row r="10" spans="1:7" s="5" customFormat="1" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
@@ -2720,7 +2720,7 @@
       <c r="F10" s="4"/>
       <c r="G10" s="7"/>
     </row>
-    <row r="11" spans="1:7" s="5" customFormat="1" ht="134.4">
+    <row r="11" spans="1:7" s="5" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>50</v>
       </c>
@@ -2739,7 +2739,7 @@
       <c r="F11" s="4"/>
       <c r="G11" s="7"/>
     </row>
-    <row r="12" spans="1:7" s="5" customFormat="1" ht="100.8">
+    <row r="12" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>55</v>
       </c>
@@ -2758,7 +2758,7 @@
       <c r="F12" s="4"/>
       <c r="G12" s="7"/>
     </row>
-    <row r="13" spans="1:7" s="5" customFormat="1" ht="117.6">
+    <row r="13" spans="1:7" s="5" customFormat="1" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>60</v>
       </c>
@@ -2777,7 +2777,7 @@
       <c r="F13" s="4"/>
       <c r="G13" s="7"/>
     </row>
-    <row r="14" spans="1:7" s="5" customFormat="1" ht="117.6">
+    <row r="14" spans="1:7" s="5" customFormat="1" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>65</v>
       </c>
@@ -2796,7 +2796,7 @@
       <c r="F14" s="4"/>
       <c r="G14" s="7"/>
     </row>
-    <row r="15" spans="1:7" s="5" customFormat="1" ht="117.6">
+    <row r="15" spans="1:7" s="5" customFormat="1" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>70</v>
       </c>
@@ -2824,41 +2824,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2740FEBB-4741-4DF0-A699-0C7B375BBE03}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{168DB4B3-5DF8-4A41-93E0-CE7F8314E965}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6E890A5-A39F-47F1-9197-F34001BFD460}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="16.8"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.19921875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="22.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.59765625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="23.19921875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.8984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.8984375" style="1"/>
+    <col min="1" max="1" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.21875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>75</v>
       </c>
@@ -2881,7 +2861,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="50.4">
+    <row r="2" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
         <v>5</v>
       </c>
@@ -2904,7 +2884,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="67.2">
+    <row r="3" spans="1:7" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -2927,7 +2907,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="50.4">
+    <row r="4" spans="1:7" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
         <v>15</v>
       </c>
@@ -2950,7 +2930,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2958,7 +2938,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="33.6">
+    <row r="6" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>25</v>
       </c>
@@ -2966,7 +2946,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
@@ -2974,7 +2954,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="33.6">
+    <row r="8" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>35</v>
       </c>
@@ -2982,7 +2962,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="33.6">
+    <row r="9" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
@@ -2990,7 +2970,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="33.6">
+    <row r="10" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>45</v>
       </c>
@@ -2998,7 +2978,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>50</v>
       </c>
@@ -3006,7 +2986,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>55</v>
       </c>
@@ -3014,7 +2994,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="33.6">
+    <row r="13" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -3022,7 +3002,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="33.6">
+    <row r="14" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>65</v>
       </c>
@@ -3030,7 +3010,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="33.6">
+    <row r="15" spans="1:7" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>70</v>
       </c>
@@ -3051,22 +3031,42 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2740FEBB-4741-4DF0-A699-0C7B375BBE03}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{168DB4B3-5DF8-4A41-93E0-CE7F8314E965}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED1CF396-0CEE-423B-9F0A-D9AA10B67D4E}">
   <dimension ref="A5:A82"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="5" spans="1:1" ht="24.6">
+    <row r="5" spans="1:1" ht="24.6" x14ac:dyDescent="0.4">
       <c r="A5" s="18" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="24.6">
+    <row r="23" spans="1:1" ht="25.8" x14ac:dyDescent="0.5">
       <c r="A23" s="19" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="82" spans="1:1" ht="24.6">
+    <row r="82" spans="1:1" ht="24.6" x14ac:dyDescent="0.4">
       <c r="A82" s="18" t="s">
         <v>86</v>
       </c>

</xml_diff>